<commit_message>
Add local Streamlit web UI, background jobs, and v0.2 pipeline.
Introduces app/ for localhost-only operations, ops SQLite layer, script renumbering, and updated ops priority rules.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/outputs/reports/catboost/evaluation.xlsx
+++ b/outputs/reports/catboost/evaluation.xlsx
@@ -487,37 +487,37 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.9906432546403512</v>
+        <v>0.9893713857357036</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2136498516320475</v>
+        <v>0.222541690626797</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9266409266409267</v>
+        <v>0.911660777385159</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3472389679286231</v>
+        <v>0.35775363993529</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9908156086132263</v>
+        <v>0.9896245419488517</v>
       </c>
       <c r="G2" t="n">
-        <v>285883</v>
+        <v>257911</v>
       </c>
       <c r="H2" t="n">
-        <v>2650</v>
+        <v>2704</v>
       </c>
       <c r="I2" t="n">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="J2" t="n">
-        <v>720</v>
+        <v>774</v>
       </c>
       <c r="K2" t="n">
-        <v>0.9762611907184625</v>
+        <v>0.9860349941936518</v>
       </c>
       <c r="L2" t="n">
-        <v>0.6669118333811218</v>
+        <v>0.6974527412588878</v>
       </c>
     </row>
   </sheetData>
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -562,32 +562,47 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>상위1%양성포착비율(top_1pct_recall)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>상위5%건수(top_5pct_count)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>상위5%양성비율(top_5pct_positive_rate)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>상위5%리프트(top_5pct_lift)</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>상위5%양성포착비율(top_5pct_recall)</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
         <is>
           <t>상위10%건수(top_10pct_count)</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>상위10%양성비율(top_10pct_positive_rate)</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>상위10%리프트(top_10pct_lift)</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>상위10%양성포착비율(top_10pct_recall)</t>
         </is>
       </c>
     </row>
@@ -598,34 +613,43 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.002685700459714493</v>
+        <v>0.003247100939326255</v>
       </c>
       <c r="C2" t="n">
-        <v>2894</v>
+        <v>2615</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2460262612301313</v>
+        <v>0.2860420650095603</v>
       </c>
       <c r="E2" t="n">
-        <v>91.60599438415609</v>
+        <v>88.09152236237887</v>
       </c>
       <c r="F2" t="n">
-        <v>14466</v>
+        <v>0.8810365135453475</v>
       </c>
       <c r="G2" t="n">
-        <v>0.05087792064150422</v>
+        <v>13074</v>
       </c>
       <c r="H2" t="n">
-        <v>18.94400414516549</v>
+        <v>0.06218448829738412</v>
       </c>
       <c r="I2" t="n">
-        <v>28931</v>
+        <v>19.15077155263515</v>
       </c>
       <c r="J2" t="n">
-        <v>0.02547440461788393</v>
+        <v>0.9575971731448764</v>
       </c>
       <c r="K2" t="n">
-        <v>9.485199485199486</v>
+        <v>26147</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.03147588633495239</v>
+      </c>
+      <c r="M2" t="n">
+        <v>9.693534917175489</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.9693757361601885</v>
       </c>
     </row>
   </sheetData>
@@ -676,13 +700,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>223656</v>
+        <v>208751</v>
       </c>
       <c r="C2" t="n">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0001386057159208785</v>
+        <v>9.580792427341666e-05</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -695,13 +719,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>44036</v>
+        <v>33069</v>
       </c>
       <c r="C3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0002270869288763739</v>
+        <v>0.000272158214642112</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -714,13 +738,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>13304</v>
+        <v>10446</v>
       </c>
       <c r="C4" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0004509921828021648</v>
+        <v>0.001148765077541643</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -733,13 +757,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3621</v>
+        <v>3979</v>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="D5" t="n">
-        <v>0.001104667219000276</v>
+        <v>0.004021110831867303</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -752,13 +776,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1315</v>
+        <v>1734</v>
       </c>
       <c r="C6" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="D6" t="n">
-        <v>0.004562737642585551</v>
+        <v>0.01038062283737024</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -771,13 +795,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>661</v>
+        <v>805</v>
       </c>
       <c r="C7" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0151285930408472</v>
+        <v>0.02608695652173913</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -790,13 +814,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>501</v>
+        <v>529</v>
       </c>
       <c r="C8" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="D8" t="n">
-        <v>0.02594810379241517</v>
+        <v>0.03402646502835539</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -809,13 +833,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>520</v>
+        <v>446</v>
       </c>
       <c r="C9" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D9" t="n">
-        <v>0.04423076923076923</v>
+        <v>0.04708520179372197</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -828,13 +852,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>433</v>
+        <v>455</v>
       </c>
       <c r="C10" t="n">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="D10" t="n">
-        <v>0.05080831408775981</v>
+        <v>0.1010989010989011</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -847,13 +871,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1263</v>
+        <v>1250</v>
       </c>
       <c r="C11" t="n">
-        <v>652</v>
+        <v>668</v>
       </c>
       <c r="D11" t="n">
-        <v>0.5162311955661124</v>
+        <v>0.5344</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>

</xml_diff>